<commit_message>
Adiciona SB LOG ao fechamento e torna o casamento por EAN determinístico
SB LOG devolve a RFQ com coluna Estoque SB: 127 itens cotados, 14 no
pedido (R$ 1.753,14). Casamento por EAN passa a priorizar o EAN
principal em ordem estável (antes dependia da ordem de um set,
variando entre execuções). Fechamento: 10 pedidos, 905 itens,
R$ 73.298,52; OL × pedidos = 0.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VLivvbyTHZf5HaiMxTfGPo
</commit_message>
<xml_diff>
--- a/cotacoes/2026-09-08/fechamento/PEDIDO_TAPAJOS_09-09-2026.xlsx
+++ b/cotacoes/2026-09-08/fechamento/PEDIDO_TAPAJOS_09-09-2026.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q93"/>
+  <dimension ref="A1:Q92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1225,30 +1225,30 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>588821</v>
+        <v>666671</v>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>7891106912167</t>
+          <t>7891106914628</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>BEPANTOL BABY 30+15G</t>
+          <t>BEPANTOL DERMA REGENERADOR 200ML-DEMAIS PROD</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>14.83</v>
+        <v>46.5</v>
       </c>
       <c r="I13" s="5">
         <f>G13*H13</f>
@@ -1259,13 +1259,13 @@
         <v/>
       </c>
       <c r="K13" s="5" t="n">
-        <v>14.36</v>
+        <v>59.3</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>12.9012</v>
+        <v>59.3</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>13.7404</v>
+        <v>59.29999999999999</v>
       </c>
       <c r="N13" s="6">
         <f>J13/M13-1</f>
@@ -1277,37 +1277,37 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +3.3% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>666671</v>
+        <v>31103</v>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>7891106914628</t>
+          <t>7896714296418</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BEPANTOL DERMA REGENERADOR 200ML-DEMAIS PROD</t>
+          <t>BETAM+DIPR FOS 5MG/ML C/1APX1ML (NQG)</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>46.5</v>
+        <v>5.76</v>
       </c>
       <c r="I14" s="5">
         <f>G14*H14</f>
@@ -1318,13 +1318,13 @@
         <v/>
       </c>
       <c r="K14" s="5" t="n">
-        <v>59.3</v>
+        <v>6.37</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>59.3</v>
+        <v>5.76</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>59.29999999999999</v>
+        <v>5.760000000000001</v>
       </c>
       <c r="N14" s="6">
         <f>J14/M14-1</f>
@@ -1343,30 +1343,30 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>31103</v>
+        <v>254101</v>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>7896714296418</t>
+          <t>7891317103323</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>BETAM+DIPR FOS 5MG/ML C/1APX1ML (NQG)</t>
+          <t>BETATRINTA 5+2MG/ML SUS INJ AMP X 1ML+SER SIST</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>5.76</v>
+        <v>22.91</v>
       </c>
       <c r="I15" s="5">
         <f>G15*H15</f>
@@ -1377,13 +1377,13 @@
         <v/>
       </c>
       <c r="K15" s="5" t="n">
-        <v>6.37</v>
+        <v>22.91</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>5.76</v>
+        <v>20.871</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>5.760000000000001</v>
+        <v>22.147</v>
       </c>
       <c r="N15" s="6">
         <f>J15/M15-1</f>
@@ -1402,30 +1402,30 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>254101</v>
+        <v>128081</v>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>7891317103323</t>
+          <t>7891317478964</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>BETATRINTA 5+2MG/ML SUS INJ AMP X 1ML+SER SIST</t>
+          <t>BETINA 24MG CX 30 COMP</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>22.91</v>
+        <v>28.76</v>
       </c>
       <c r="I16" s="5">
         <f>G16*H16</f>
@@ -1436,13 +1436,13 @@
         <v/>
       </c>
       <c r="K16" s="5" t="n">
-        <v>22.91</v>
+        <v>29.58</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>20.871</v>
+        <v>26.87</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>22.147</v>
+        <v>28.17333333333333</v>
       </c>
       <c r="N16" s="6">
         <f>J16/M16-1</f>
@@ -1461,17 +1461,17 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>128081</v>
+        <v>550721</v>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>7891317478964</t>
+          <t>7891317001964</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>BETINA 24MG CX 30 COMP</t>
+          <t>BICERTO 150MG CX 10 COMP LIB PROL</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1484,7 +1484,7 @@
         <v>3</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>28.76</v>
+        <v>40.07</v>
       </c>
       <c r="I17" s="5">
         <f>G17*H17</f>
@@ -1495,13 +1495,13 @@
         <v/>
       </c>
       <c r="K17" s="5" t="n">
-        <v>29.58</v>
+        <v>41.2</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>26.87</v>
+        <v>36.52</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>28.17333333333333</v>
+        <v>38.74666666666667</v>
       </c>
       <c r="N17" s="6">
         <f>J17/M17-1</f>
@@ -1520,30 +1520,30 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>550721</v>
+        <v>114841</v>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>7891317001964</t>
+          <t>7892953003527</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>BICERTO 150MG CX 10 COMP LIB PROL</t>
+          <t>BIO-VAGIN 62,5+1,25MG+25.000UI/G CREM VAG BG 40G+10APL</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>40.07</v>
+        <v>58.74</v>
       </c>
       <c r="I18" s="5">
         <f>G18*H18</f>
@@ -1554,13 +1554,13 @@
         <v/>
       </c>
       <c r="K18" s="5" t="n">
-        <v>41.2</v>
+        <v>61.69</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>36.52</v>
+        <v>54.79</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>38.74666666666667</v>
+        <v>58.31</v>
       </c>
       <c r="N18" s="6">
         <f>J18/M18-1</f>
@@ -1579,30 +1579,30 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>114841</v>
+        <v>293601</v>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>7892953003527</t>
+          <t>7896548140284</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>BIO-VAGIN 62,5+1,25MG+25.000UI/G CREM VAG BG 40G+10APL</t>
+          <t>CERUMIN 0,4+140MG SOL OTO FR GTS 8ML</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>58.74</v>
+        <v>21.23</v>
       </c>
       <c r="I19" s="5">
         <f>G19*H19</f>
@@ -1613,13 +1613,13 @@
         <v/>
       </c>
       <c r="K19" s="5" t="n">
-        <v>61.69</v>
+        <v>21.23</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>54.79</v>
+        <v>13.7043</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>58.31</v>
+        <v>17.67023333333333</v>
       </c>
       <c r="N19" s="6">
         <f>J19/M19-1</f>
@@ -1638,30 +1638,30 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>293601</v>
+        <v>135661</v>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>7896548140284</t>
+          <t>7891158106965</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>CERUMIN 0,4+140MG SOL OTO FR GTS 8ML</t>
+          <t>COBAVITAL 1+4MG 16 COMP</t>
         </is>
       </c>
       <c r="E20" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>21.23</v>
+        <v>21.67</v>
       </c>
       <c r="I20" s="5">
         <f>G20*H20</f>
@@ -1672,13 +1672,13 @@
         <v/>
       </c>
       <c r="K20" s="5" t="n">
-        <v>21.23</v>
+        <v>21.67</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>13.7043</v>
+        <v>18.21</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>17.67023333333333</v>
+        <v>20.20833333333334</v>
       </c>
       <c r="N20" s="6">
         <f>J20/M20-1</f>
@@ -1697,30 +1697,30 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>135661</v>
+        <v>6561</v>
       </c>
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>7891158106965</t>
+          <t>7894916502900</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>COBAVITAL 1+4MG 16 COMP</t>
+          <t>CONTRACEP SUS INJ 1 FA X 1ML</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>21.67</v>
+        <v>23.94</v>
       </c>
       <c r="I21" s="5">
         <f>G21*H21</f>
@@ -1731,13 +1731,13 @@
         <v/>
       </c>
       <c r="K21" s="5" t="n">
-        <v>21.67</v>
+        <v>23.69</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>18.21</v>
+        <v>22.9</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>20.20833333333334</v>
+        <v>23.16333333333334</v>
       </c>
       <c r="N21" s="6">
         <f>J21/M21-1</f>
@@ -1749,37 +1749,37 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6561</v>
+        <v>90721</v>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>7894916502900</t>
+          <t>7891317137557</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>CONTRACEP SUS INJ 1 FA X 1ML</t>
+          <t>COQUES 200MG CX 10 CAP</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>23.94</v>
+        <v>33.84</v>
       </c>
       <c r="I22" s="5">
         <f>G22*H22</f>
@@ -1790,13 +1790,13 @@
         <v/>
       </c>
       <c r="K22" s="5" t="n">
-        <v>23.69</v>
+        <v>34.79</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>22.9</v>
+        <v>30.618</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>23.16333333333334</v>
+        <v>32.46266666666666</v>
       </c>
       <c r="N22" s="6">
         <f>J22/M22-1</f>
@@ -1808,37 +1808,37 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>90721</v>
+        <v>463461</v>
       </c>
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>7891317137557</t>
+          <t>7891317136468</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>COQUES 200MG CX 10 CAP</t>
+          <t>CREVAGIN 30+20MG CREM VAG BG X 40G +7APLIC</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>33.84</v>
+        <v>38.8</v>
       </c>
       <c r="I23" s="5">
         <f>G23*H23</f>
@@ -1849,13 +1849,13 @@
         <v/>
       </c>
       <c r="K23" s="5" t="n">
-        <v>34.79</v>
+        <v>38.8</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>30.618</v>
+        <v>35.79</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>32.46266666666666</v>
+        <v>37.32443333333333</v>
       </c>
       <c r="N23" s="6">
         <f>J23/M23-1</f>
@@ -1874,30 +1874,30 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>463461</v>
+        <v>821</v>
       </c>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>7891317136468</t>
+          <t>7893454100661</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>CREVAGIN 30+20MG CREM VAG BG X 40G +7APLIC</t>
+          <t>DERMOSALIC 30G POM BG</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>38.8</v>
+        <v>10.46</v>
       </c>
       <c r="I24" s="5">
         <f>G24*H24</f>
@@ -1908,13 +1908,13 @@
         <v/>
       </c>
       <c r="K24" s="5" t="n">
-        <v>38.8</v>
+        <v>10.36</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>35.79</v>
+        <v>10.36</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>37.32443333333333</v>
+        <v>10.36</v>
       </c>
       <c r="N24" s="6">
         <f>J24/M24-1</f>
@@ -1926,37 +1926,37 @@
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.0% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>821</v>
+        <v>341641</v>
       </c>
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>7893454100661</t>
+          <t>7891317455569</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>DERMOSALIC 30G POM BG</t>
+          <t>DUOMO 2MG CX 30 COMP</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>10.46</v>
+        <v>30.95</v>
       </c>
       <c r="I25" s="5">
         <f>G25*H25</f>
@@ -1967,13 +1967,13 @@
         <v/>
       </c>
       <c r="K25" s="5" t="n">
-        <v>10.36</v>
+        <v>30.62</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>10.36</v>
+        <v>28.95</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>10.36</v>
+        <v>30.06333333333333</v>
       </c>
       <c r="N25" s="6">
         <f>J25/M25-1</f>
@@ -1985,37 +1985,37 @@
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.0% vs últ. (≤4%)</t>
+          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>341641</v>
+        <v>15</v>
       </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>7891317455569</t>
+          <t>7896094903272</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>DUOMO 2MG CX 30 COMP</t>
+          <t>EPOCLER SOL ORAL FLACONETE CAIXA C/ 12</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>30.95</v>
+        <v>35.68</v>
       </c>
       <c r="I26" s="5">
         <f>G26*H26</f>
@@ -2025,56 +2025,44 @@
         <f>H26/E26</f>
         <v/>
       </c>
-      <c r="K26" s="5" t="n">
-        <v>30.62</v>
-      </c>
-      <c r="L26" s="5" t="n">
-        <v>28.95</v>
-      </c>
-      <c r="M26" s="5" t="n">
-        <v>30.06333333333333</v>
-      </c>
-      <c r="N26" s="6">
-        <f>J26/M26-1</f>
-        <v/>
-      </c>
-      <c r="O26" s="6">
-        <f>J26/K26-1</f>
-        <v/>
-      </c>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="5" t="n"/>
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="6" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
+          <t>SEM HISTÓRICO</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>15</v>
+        <v>623691</v>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>7896094903272</t>
+          <t>7896714274423</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>EPOCLER SOL ORAL FLACONETE CAIXA C/ 12</t>
+          <t>EQUILIBRISSE 420MG CX 10 COMP REV</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>35.68</v>
+        <v>9.81</v>
       </c>
       <c r="I27" s="5">
         <f>G27*H27</f>
@@ -2084,44 +2072,56 @@
         <f>H27/E27</f>
         <v/>
       </c>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
-      <c r="M27" s="5" t="n"/>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="6" t="n"/>
+      <c r="K27" s="5" t="n">
+        <v>9.81</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>9.726666666666667</v>
+      </c>
+      <c r="N27" s="6">
+        <f>J27/M27-1</f>
+        <v/>
+      </c>
+      <c r="O27" s="6">
+        <f>J27/K27-1</f>
+        <v/>
+      </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>SEM HISTÓRICO</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>623691</v>
+        <v>582241</v>
       </c>
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>7896714274423</t>
+          <t>7896637031943</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>EQUILIBRISSE 420MG CX 10 COMP REV</t>
+          <t>FLANCOX 600MG CX 14 REV OR</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>9.81</v>
+        <v>46.73999999999999</v>
       </c>
       <c r="I28" s="5">
         <f>G28*H28</f>
@@ -2132,13 +2132,13 @@
         <v/>
       </c>
       <c r="K28" s="5" t="n">
-        <v>9.81</v>
+        <v>47.24</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>9.56</v>
+        <v>43.5075</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>9.726666666666667</v>
+        <v>45.21806666666667</v>
       </c>
       <c r="N28" s="6">
         <f>J28/M28-1</f>
@@ -2157,30 +2157,30 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>582241</v>
+        <v>589581</v>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>7896637031943</t>
+          <t>7898040329655</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>FLANCOX 600MG CX 14 REV OR</t>
+          <t>FLORATIL 200MG CX 6 CAP</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>46.73999999999999</v>
+        <v>36.79</v>
       </c>
       <c r="I29" s="5">
         <f>G29*H29</f>
@@ -2191,13 +2191,13 @@
         <v/>
       </c>
       <c r="K29" s="5" t="n">
-        <v>47.24</v>
+        <v>37.185</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>43.5075</v>
+        <v>27.3967</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>45.21806666666667</v>
+        <v>33.92056666666667</v>
       </c>
       <c r="N29" s="6">
         <f>J29/M29-1</f>
@@ -2216,17 +2216,17 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>589581</v>
+        <v>589611</v>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>7898040329655</t>
+          <t>7898040329570</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>FLORATIL 200MG CX 6 CAP</t>
+          <t>FLORATIL 200MG/G PO OR 4 ENV X 1G</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
@@ -2239,7 +2239,7 @@
         <v>6</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>36.79</v>
+        <v>28.2</v>
       </c>
       <c r="I30" s="5">
         <f>G30*H30</f>
@@ -2250,13 +2250,13 @@
         <v/>
       </c>
       <c r="K30" s="5" t="n">
-        <v>37.185</v>
+        <v>28</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>27.3967</v>
+        <v>7.05</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>33.92056666666667</v>
+        <v>7.05</v>
       </c>
       <c r="N30" s="6">
         <f>J30/M30-1</f>
@@ -2268,37 +2268,37 @@
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>589611</v>
+        <v>622951</v>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>7898040329570</t>
+          <t>7898040329679</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>FLORATIL 200MG/G PO OR 4 ENV X 1G</t>
+          <t>FLORATIL 250MG BL 6 CAP</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>28.2</v>
+        <v>36.79</v>
       </c>
       <c r="I31" s="5">
         <f>G31*H31</f>
@@ -2309,13 +2309,13 @@
         <v/>
       </c>
       <c r="K31" s="5" t="n">
-        <v>28</v>
+        <v>38.6417</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>7.05</v>
+        <v>31.31</v>
       </c>
       <c r="M31" s="5" t="n">
-        <v>7.05</v>
+        <v>33.75333333333334</v>
       </c>
       <c r="N31" s="6">
         <f>J31/M31-1</f>
@@ -2327,34 +2327,34 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>622951</v>
+        <v>671851</v>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>7898040329679</t>
+          <t>7898040329600</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>FLORATIL 250MG BL 6 CAP</t>
+          <t>FLORATIL 250MG BL 6 SACHE</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H32" s="5" t="n">
         <v>36.79</v>
@@ -2368,13 +2368,13 @@
         <v/>
       </c>
       <c r="K32" s="5" t="n">
-        <v>38.6417</v>
+        <v>36.79</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>31.31</v>
+        <v>30.505</v>
       </c>
       <c r="M32" s="5" t="n">
-        <v>33.75333333333334</v>
+        <v>34.695</v>
       </c>
       <c r="N32" s="6">
         <f>J32/M32-1</f>
@@ -2393,30 +2393,30 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>671851</v>
+        <v>636341</v>
       </c>
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>7898040329600</t>
+          <t>7891317023331</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>FLORATIL 250MG BL 6 SACHE</t>
+          <t>FORFIG 200MG CX 20 CAP</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>36.79</v>
+        <v>112.26</v>
       </c>
       <c r="I33" s="5">
         <f>G33*H33</f>
@@ -2427,13 +2427,13 @@
         <v/>
       </c>
       <c r="K33" s="5" t="n">
-        <v>36.79</v>
+        <v>115.42</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>30.505</v>
+        <v>102.85</v>
       </c>
       <c r="M33" s="5" t="n">
-        <v>34.695</v>
+        <v>111.23</v>
       </c>
       <c r="N33" s="6">
         <f>J33/M33-1</f>
@@ -2452,30 +2452,30 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>636341</v>
+        <v>36003</v>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>7891317023331</t>
+          <t>7896714296500</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>FORFIG 200MG CX 20 CAP</t>
+          <t>FUROATO DE MOMETASONA 0,5MG/G SPRAY NAS 120 DOSES</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>112.26</v>
+        <v>25.01</v>
       </c>
       <c r="I34" s="5">
         <f>G34*H34</f>
@@ -2486,13 +2486,13 @@
         <v/>
       </c>
       <c r="K34" s="5" t="n">
-        <v>115.42</v>
+        <v>25.88</v>
       </c>
       <c r="L34" s="5" t="n">
-        <v>102.85</v>
+        <v>25.88</v>
       </c>
       <c r="M34" s="5" t="n">
-        <v>111.23</v>
+        <v>25.88</v>
       </c>
       <c r="N34" s="6">
         <f>J34/M34-1</f>
@@ -2511,30 +2511,30 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>36003</v>
+        <v>36103</v>
       </c>
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>7896714296500</t>
+          <t>7896714296494</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>FUROATO DE MOMETASONA 0,5MG/G SPRAY NAS 120 DOSES</t>
+          <t>FUROATO DE MOMETASONA 0,5MG/G SPRAY NAS 60 DOSES</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>25.01</v>
+        <v>17.95</v>
       </c>
       <c r="I35" s="5">
         <f>G35*H35</f>
@@ -2545,13 +2545,13 @@
         <v/>
       </c>
       <c r="K35" s="5" t="n">
-        <v>25.88</v>
+        <v>19.83</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>25.88</v>
+        <v>19.83</v>
       </c>
       <c r="M35" s="5" t="n">
-        <v>25.88</v>
+        <v>19.83</v>
       </c>
       <c r="N35" s="6">
         <f>J35/M35-1</f>
@@ -2570,30 +2570,30 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>36103</v>
+        <v>660241</v>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>7896714296494</t>
+          <t>7896862993665</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>FUROATO DE MOMETASONA 0,5MG/G SPRAY NAS 60 DOSES</t>
+          <t>GASTROGEL TABS MENTA (CARTELA)</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>17.95</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="I36" s="5">
         <f>G36*H36</f>
@@ -2604,13 +2604,13 @@
         <v/>
       </c>
       <c r="K36" s="5" t="n">
-        <v>19.83</v>
+        <v>7.99</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>19.83</v>
+        <v>7.99</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>19.83</v>
+        <v>7.989999999999999</v>
       </c>
       <c r="N36" s="6">
         <f>J36/M36-1</f>
@@ -2622,24 +2622,24 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +5.9% vs média (≤6%)</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>660241</v>
+        <v>635741</v>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>7896862993665</t>
+          <t>7891106916059</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>GASTROGEL TABS MENTA (CARTELA)</t>
+          <t>GINO CANESTEN 1 500MG 1COMP+APL-REFERENCIA</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -2652,7 +2652,7 @@
         <v>4</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>8.460000000000001</v>
+        <v>78.02</v>
       </c>
       <c r="I37" s="5">
         <f>G37*H37</f>
@@ -2663,13 +2663,13 @@
         <v/>
       </c>
       <c r="K37" s="5" t="n">
-        <v>7.99</v>
+        <v>80.51000000000001</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>7.99</v>
+        <v>68.87</v>
       </c>
       <c r="M37" s="5" t="n">
-        <v>7.989999999999999</v>
+        <v>71.25666666666667</v>
       </c>
       <c r="N37" s="6">
         <f>J37/M37-1</f>
@@ -2681,37 +2681,37 @@
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +5.9% vs média (≤6%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>635741</v>
+        <v>36203</v>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>7891106916059</t>
+          <t>7896714294520</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>GINO CANESTEN 1 500MG 1COMP+APL-REFERENCIA</t>
+          <t>GLICLAZIDA 30MG 30 CPR LIB PROL</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>78.02</v>
+        <v>7.56</v>
       </c>
       <c r="I38" s="5">
         <f>G38*H38</f>
@@ -2722,13 +2722,13 @@
         <v/>
       </c>
       <c r="K38" s="5" t="n">
-        <v>80.51000000000001</v>
+        <v>7.15</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>68.87</v>
+        <v>7.15</v>
       </c>
       <c r="M38" s="5" t="n">
-        <v>71.25666666666667</v>
+        <v>7.150000000000001</v>
       </c>
       <c r="N38" s="6">
         <f>J38/M38-1</f>
@@ -2740,37 +2740,37 @@
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +5.7% vs média (≤6%)</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>36203</v>
+        <v>264141</v>
       </c>
       <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>7896714294520</t>
+          <t>7891721026621</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>GLICLAZIDA 30MG 30 CPR LIB PROL</t>
+          <t>GLUCOVANCE 500+5MG CX 30 COMP REV</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>7.56</v>
+        <v>40.76</v>
       </c>
       <c r="I39" s="5">
         <f>G39*H39</f>
@@ -2781,13 +2781,13 @@
         <v/>
       </c>
       <c r="K39" s="5" t="n">
-        <v>7.15</v>
+        <v>42.8067</v>
       </c>
       <c r="L39" s="5" t="n">
-        <v>7.15</v>
+        <v>40.76</v>
       </c>
       <c r="M39" s="5" t="n">
-        <v>7.150000000000001</v>
+        <v>40.76</v>
       </c>
       <c r="N39" s="6">
         <f>J39/M39-1</f>
@@ -2799,37 +2799,37 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +5.7% vs média (≤6%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>264141</v>
+        <v>213481</v>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>7891721026621</t>
+          <t>7897129301506</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>GLUCOVANCE 500+5MG CX 30 COMP REV</t>
+          <t>HIXIZINE 2MG/ML SOL OR FR 120ML</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>40.76</v>
+        <v>47.38</v>
       </c>
       <c r="I40" s="5">
         <f>G40*H40</f>
@@ -2840,13 +2840,13 @@
         <v/>
       </c>
       <c r="K40" s="5" t="n">
-        <v>42.8067</v>
+        <v>47.88</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>40.76</v>
+        <v>43.2</v>
       </c>
       <c r="M40" s="5" t="n">
-        <v>40.76</v>
+        <v>45.56890000000001</v>
       </c>
       <c r="N40" s="6">
         <f>J40/M40-1</f>
@@ -2865,17 +2865,17 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>213481</v>
+        <v>14103</v>
       </c>
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>7897129301506</t>
+          <t>7899620913202</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>HIXIZINE 2MG/ML SOL OR FR 120ML</t>
+          <t>KALOSTOP (N.S.) 0,20+0,15ML/ML SOL FR 10ML</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
@@ -2888,7 +2888,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>47.38</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="I41" s="5">
         <f>G41*H41</f>
@@ -2899,13 +2899,13 @@
         <v/>
       </c>
       <c r="K41" s="5" t="n">
-        <v>47.88</v>
+        <v>8.41</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>43.2</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="M41" s="5" t="n">
-        <v>45.56890000000001</v>
+        <v>8.376666666666667</v>
       </c>
       <c r="N41" s="6">
         <f>J41/M41-1</f>
@@ -2917,37 +2917,37 @@
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +2.7% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>14103</v>
+        <v>190241</v>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>7899620913202</t>
+          <t>7896676427745</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>KALOSTOP (N.S.) 0,20+0,15ML/ML SOL FR 10ML</t>
+          <t>KOLLAGENASE 0,6U/G POM DERM BG 30G+ESP</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>8.640000000000001</v>
+        <v>54.36</v>
       </c>
       <c r="I42" s="5">
         <f>G42*H42</f>
@@ -2958,13 +2958,13 @@
         <v/>
       </c>
       <c r="K42" s="5" t="n">
-        <v>8.41</v>
+        <v>54.35</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>8.359999999999999</v>
+        <v>49.1033</v>
       </c>
       <c r="M42" s="5" t="n">
-        <v>8.376666666666667</v>
+        <v>51.83276666666666</v>
       </c>
       <c r="N42" s="6">
         <f>J42/M42-1</f>
@@ -2976,37 +2976,37 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +2.7% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>190241</v>
+        <v>114101</v>
       </c>
       <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>7896676427745</t>
+          <t>7896676427844</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>KOLLAGENASE 0,6U/G POM DERM BG 30G+ESP</t>
+          <t>KOLLAGENASE+CLORANFENICOL 0,6U/G+0,01G/G POM DERM BG 15G+ESP</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>54.36</v>
+        <v>27.55</v>
       </c>
       <c r="I43" s="5">
         <f>G43*H43</f>
@@ -3017,13 +3017,13 @@
         <v/>
       </c>
       <c r="K43" s="5" t="n">
-        <v>54.35</v>
+        <v>29.24</v>
       </c>
       <c r="L43" s="5" t="n">
-        <v>49.1033</v>
+        <v>25.52</v>
       </c>
       <c r="M43" s="5" t="n">
-        <v>51.83276666666666</v>
+        <v>26.78333333333333</v>
       </c>
       <c r="N43" s="6">
         <f>J43/M43-1</f>
@@ -3035,37 +3035,37 @@
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>114101</v>
+        <v>208201</v>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>7896676427844</t>
+          <t>7896676432855</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>KOLLAGENASE+CLORANFENICOL 0,6U/G+0,01G/G POM DERM BG 15G+ESP</t>
+          <t>LACRIBELL 1+3MG SOL OFT FR 15ML</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>27.55</v>
+        <v>18.59</v>
       </c>
       <c r="I44" s="5">
         <f>G44*H44</f>
@@ -3076,13 +3076,13 @@
         <v/>
       </c>
       <c r="K44" s="5" t="n">
-        <v>29.24</v>
+        <v>19.53</v>
       </c>
       <c r="L44" s="5" t="n">
-        <v>25.52</v>
+        <v>17.415</v>
       </c>
       <c r="M44" s="5" t="n">
-        <v>26.78333333333333</v>
+        <v>18.48</v>
       </c>
       <c r="N44" s="6">
         <f>J44/M44-1</f>
@@ -3101,30 +3101,30 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>208201</v>
+        <v>549281</v>
       </c>
       <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>7896676432855</t>
+          <t>7896004768465</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>LACRIBELL 1+3MG SOL OFT FR 15ML</t>
+          <t>LACTULIV 667MG/ML 120ML AMEIXA (LACTULOS</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H45" s="5" t="n">
-        <v>18.59</v>
+        <v>11.33</v>
       </c>
       <c r="I45" s="5">
         <f>G45*H45</f>
@@ -3135,13 +3135,13 @@
         <v/>
       </c>
       <c r="K45" s="5" t="n">
-        <v>19.53</v>
+        <v>13.43</v>
       </c>
       <c r="L45" s="5" t="n">
-        <v>17.415</v>
+        <v>12.89</v>
       </c>
       <c r="M45" s="5" t="n">
-        <v>18.48</v>
+        <v>13.07</v>
       </c>
       <c r="N45" s="6">
         <f>J45/M45-1</f>
@@ -3160,30 +3160,30 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>549281</v>
+        <v>560241</v>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>7896004768465</t>
+          <t>7894164008209</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>LACTULIV 667MG/ML 120ML AMEIXA (LACTULOS</t>
+          <t>LEFLORA 6 CAP</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H46" s="5" t="n">
-        <v>11.33</v>
+        <v>8.94</v>
       </c>
       <c r="I46" s="5">
         <f>G46*H46</f>
@@ -3194,13 +3194,13 @@
         <v/>
       </c>
       <c r="K46" s="5" t="n">
-        <v>13.43</v>
+        <v>10.42</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>12.89</v>
+        <v>10.03</v>
       </c>
       <c r="M46" s="5" t="n">
-        <v>13.07</v>
+        <v>10.29</v>
       </c>
       <c r="N46" s="6">
         <f>J46/M46-1</f>
@@ -3219,17 +3219,17 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>560241</v>
+        <v>320361</v>
       </c>
       <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>7894164008209</t>
+          <t>7896658008849</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>LEFLORA 6 CAP</t>
+          <t>LEVOID 112MCG CX 30 COMP</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
@@ -3242,7 +3242,7 @@
         <v>1</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>8.94</v>
+        <v>24.24</v>
       </c>
       <c r="I47" s="5">
         <f>G47*H47</f>
@@ -3253,13 +3253,13 @@
         <v/>
       </c>
       <c r="K47" s="5" t="n">
-        <v>10.42</v>
+        <v>23.94</v>
       </c>
       <c r="L47" s="5" t="n">
-        <v>10.03</v>
+        <v>23.94</v>
       </c>
       <c r="M47" s="5" t="n">
-        <v>10.29</v>
+        <v>23.94</v>
       </c>
       <c r="N47" s="6">
         <f>J47/M47-1</f>
@@ -3271,37 +3271,37 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.3% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>320361</v>
+        <v>284241</v>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>7896658008849</t>
+          <t>7896676435658</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>LEVOID 112MCG CX 30 COMP</t>
+          <t>LUNAH 1MG /ML SOL OFT FR GOT 10ML</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>24.24</v>
+        <v>40.67</v>
       </c>
       <c r="I48" s="5">
         <f>G48*H48</f>
@@ -3312,13 +3312,13 @@
         <v/>
       </c>
       <c r="K48" s="5" t="n">
-        <v>23.94</v>
+        <v>42.72</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>23.94</v>
+        <v>38.0767</v>
       </c>
       <c r="M48" s="5" t="n">
-        <v>23.94</v>
+        <v>39.66223333333333</v>
       </c>
       <c r="N48" s="6">
         <f>J48/M48-1</f>
@@ -3330,37 +3330,37 @@
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.3% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>284241</v>
+        <v>206681</v>
       </c>
       <c r="B49" s="2" t="inlineStr"/>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>7896676435658</t>
+          <t>7896548111727</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>LUNAH 1MG /ML SOL OFT FR GOT 10ML</t>
+          <t>MAXIDEX 1MG/ML SUS OFT FR GTS 5ML</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>40.67</v>
+        <v>8.27</v>
       </c>
       <c r="I49" s="5">
         <f>G49*H49</f>
@@ -3371,13 +3371,13 @@
         <v/>
       </c>
       <c r="K49" s="5" t="n">
-        <v>42.72</v>
+        <v>8.23</v>
       </c>
       <c r="L49" s="5" t="n">
-        <v>38.0767</v>
+        <v>7.8167</v>
       </c>
       <c r="M49" s="5" t="n">
-        <v>39.66223333333333</v>
+        <v>7.9889</v>
       </c>
       <c r="N49" s="6">
         <f>J49/M49-1</f>
@@ -3389,37 +3389,37 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +0.5% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>206681</v>
+        <v>337721</v>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>7896548111727</t>
+          <t>7896637023115</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>MAXIDEX 1MG/ML SUS OFT FR GTS 5ML</t>
+          <t>MECLIN 25MG CX 15 COMP</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>8.27</v>
+        <v>21.27</v>
       </c>
       <c r="I50" s="5">
         <f>G50*H50</f>
@@ -3430,13 +3430,13 @@
         <v/>
       </c>
       <c r="K50" s="5" t="n">
-        <v>8.23</v>
+        <v>21.26</v>
       </c>
       <c r="L50" s="5" t="n">
-        <v>7.8167</v>
+        <v>21.037</v>
       </c>
       <c r="M50" s="5" t="n">
-        <v>7.9889</v>
+        <v>21.11133333333333</v>
       </c>
       <c r="N50" s="6">
         <f>J50/M50-1</f>
@@ -3448,37 +3448,37 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.5% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>337721</v>
+        <v>602931</v>
       </c>
       <c r="B51" s="2" t="inlineStr"/>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>7896637023115</t>
+          <t>7896148500136</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>MECLIN 25MG CX 15 COMP</t>
+          <t>MEL CP EXTRATO PROPOLIS 35ML (FIT)</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>21.27</v>
+        <v>11.48</v>
       </c>
       <c r="I51" s="5">
         <f>G51*H51</f>
@@ -3489,13 +3489,13 @@
         <v/>
       </c>
       <c r="K51" s="5" t="n">
-        <v>21.26</v>
+        <v>11.47</v>
       </c>
       <c r="L51" s="5" t="n">
-        <v>21.037</v>
+        <v>11.47</v>
       </c>
       <c r="M51" s="5" t="n">
-        <v>21.11133333333333</v>
+        <v>11.47</v>
       </c>
       <c r="N51" s="6">
         <f>J51/M51-1</f>
@@ -3507,37 +3507,37 @@
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>602931</v>
+        <v>569961</v>
       </c>
       <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>7896148500136</t>
+          <t>7896148500709</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>MEL CP EXTRATO PROPOLIS 35ML (FIT)</t>
+          <t>MEL DE ABELHA 70G</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>11.48</v>
+        <v>6.76</v>
       </c>
       <c r="I52" s="5">
         <f>G52*H52</f>
@@ -3548,13 +3548,13 @@
         <v/>
       </c>
       <c r="K52" s="5" t="n">
-        <v>11.47</v>
+        <v>6.75</v>
       </c>
       <c r="L52" s="5" t="n">
-        <v>11.47</v>
+        <v>6.75</v>
       </c>
       <c r="M52" s="5" t="n">
-        <v>11.47</v>
+        <v>6.75</v>
       </c>
       <c r="N52" s="6">
         <f>J52/M52-1</f>
@@ -3573,17 +3573,17 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>569961</v>
+        <v>665551</v>
       </c>
       <c r="B53" s="2" t="inlineStr"/>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>7896148500709</t>
+          <t>00020800750158</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>MEL DE ABELHA 70G</t>
+          <t>METAMUCIL SOLUVEL LARANJA 174G-OUTROS</t>
         </is>
       </c>
       <c r="E53" s="4" t="n">
@@ -3596,7 +3596,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>6.76</v>
+        <v>102</v>
       </c>
       <c r="I53" s="5">
         <f>G53*H53</f>
@@ -3607,13 +3607,13 @@
         <v/>
       </c>
       <c r="K53" s="5" t="n">
-        <v>6.75</v>
+        <v>101.27</v>
       </c>
       <c r="L53" s="5" t="n">
-        <v>6.75</v>
+        <v>82.09</v>
       </c>
       <c r="M53" s="5" t="n">
-        <v>6.75</v>
+        <v>82.09</v>
       </c>
       <c r="N53" s="6">
         <f>J53/M53-1</f>
@@ -3625,37 +3625,37 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.1% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>665551</v>
+        <v>134701</v>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>00020800750158</t>
+          <t>7896637025096</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>METAMUCIL SOLUVEL LARANJA 174G-OUTROS</t>
+          <t>MIOSAN CAF 5+30MG CX 15 COMP REV</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>102</v>
+        <v>22.47</v>
       </c>
       <c r="I54" s="5">
         <f>G54*H54</f>
@@ -3666,13 +3666,13 @@
         <v/>
       </c>
       <c r="K54" s="5" t="n">
-        <v>101.27</v>
+        <v>22.71</v>
       </c>
       <c r="L54" s="5" t="n">
-        <v>82.09</v>
+        <v>19.3267</v>
       </c>
       <c r="M54" s="5" t="n">
-        <v>82.09</v>
+        <v>20.45446666666667</v>
       </c>
       <c r="N54" s="6">
         <f>J54/M54-1</f>
@@ -3684,37 +3684,37 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>134701</v>
+        <v>293561</v>
       </c>
       <c r="B55" s="2" t="inlineStr"/>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>7896637025096</t>
+          <t>7896676435214</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>MIOSAN CAF 5+30MG CX 15 COMP REV</t>
+          <t>MIRUGELL 0,4+0,3+0,1% SOL OFT FR 5ML</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>22.47</v>
+        <v>19.8</v>
       </c>
       <c r="I55" s="5">
         <f>G55*H55</f>
@@ -3725,13 +3725,13 @@
         <v/>
       </c>
       <c r="K55" s="5" t="n">
-        <v>22.71</v>
+        <v>19.8</v>
       </c>
       <c r="L55" s="5" t="n">
-        <v>19.3267</v>
+        <v>18.33</v>
       </c>
       <c r="M55" s="5" t="n">
-        <v>20.45446666666667</v>
+        <v>18.95833333333333</v>
       </c>
       <c r="N55" s="6">
         <f>J55/M55-1</f>
@@ -3750,30 +3750,30 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>293561</v>
+        <v>358341</v>
       </c>
       <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>7896676435214</t>
+          <t>7894916500296</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>MIRUGELL 0,4+0,3+0,1% SOL OFT FR 5ML</t>
+          <t>NEUTROFER 250MG SOL FR GTS 30ML</t>
         </is>
       </c>
       <c r="E56" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>19.8</v>
+        <v>47.46</v>
       </c>
       <c r="I56" s="5">
         <f>G56*H56</f>
@@ -3784,13 +3784,13 @@
         <v/>
       </c>
       <c r="K56" s="5" t="n">
-        <v>19.8</v>
+        <v>46.96</v>
       </c>
       <c r="L56" s="5" t="n">
-        <v>18.33</v>
+        <v>44.3433</v>
       </c>
       <c r="M56" s="5" t="n">
-        <v>18.95833333333333</v>
+        <v>45.21553333333333</v>
       </c>
       <c r="N56" s="6">
         <f>J56/M56-1</f>
@@ -3802,24 +3802,24 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>358341</v>
+        <v>588801</v>
       </c>
       <c r="B57" s="2" t="inlineStr"/>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>7894916500296</t>
+          <t>7898581710578</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>NEUTROFER 250MG SOL FR GTS 30ML</t>
+          <t>NORIPURUM 10MG/ML XPE FR 120ML</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
@@ -3832,7 +3832,7 @@
         <v>2</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>47.46</v>
+        <v>26.25</v>
       </c>
       <c r="I57" s="5">
         <f>G57*H57</f>
@@ -3843,13 +3843,13 @@
         <v/>
       </c>
       <c r="K57" s="5" t="n">
-        <v>46.96</v>
+        <v>26.06</v>
       </c>
       <c r="L57" s="5" t="n">
-        <v>44.3433</v>
+        <v>26.06</v>
       </c>
       <c r="M57" s="5" t="n">
-        <v>45.21553333333333</v>
+        <v>26.06</v>
       </c>
       <c r="N57" s="6">
         <f>J57/M57-1</f>
@@ -3861,37 +3861,37 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.1% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>588801</v>
+        <v>247481</v>
       </c>
       <c r="B58" s="2" t="inlineStr"/>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>7898581710578</t>
+          <t>7896641805479</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>NORIPURUM 10MG/ML XPE FR 120ML</t>
+          <t>NORIPURUM 50MG/ML SOL OR FR GOT 30ML</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>26.25</v>
+        <v>34.56</v>
       </c>
       <c r="I58" s="5">
         <f>G58*H58</f>
@@ -3902,13 +3902,13 @@
         <v/>
       </c>
       <c r="K58" s="5" t="n">
-        <v>26.06</v>
+        <v>38.21</v>
       </c>
       <c r="L58" s="5" t="n">
-        <v>26.06</v>
+        <v>34.56</v>
       </c>
       <c r="M58" s="5" t="n">
-        <v>26.06</v>
+        <v>34.56</v>
       </c>
       <c r="N58" s="6">
         <f>J58/M58-1</f>
@@ -3920,24 +3920,24 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>247481</v>
+        <v>179961</v>
       </c>
       <c r="B59" s="2" t="inlineStr"/>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>7896641805479</t>
+          <t>7898040321390</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>NORIPURUM 50MG/ML SOL OR FR GOT 30ML</t>
+          <t>OTO BETNOVATE 1+10+5MG/ML SOL OTO FR GTS 10ML</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
@@ -3950,7 +3950,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>34.56</v>
+        <v>27</v>
       </c>
       <c r="I59" s="5">
         <f>G59*H59</f>
@@ -3961,13 +3961,13 @@
         <v/>
       </c>
       <c r="K59" s="5" t="n">
-        <v>38.21</v>
+        <v>27</v>
       </c>
       <c r="L59" s="5" t="n">
-        <v>34.56</v>
+        <v>24.82</v>
       </c>
       <c r="M59" s="5" t="n">
-        <v>34.56</v>
+        <v>25.91556666666667</v>
       </c>
       <c r="N59" s="6">
         <f>J59/M59-1</f>
@@ -3986,30 +3986,30 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>179961</v>
+        <v>398941</v>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>7898040321390</t>
+          <t>7891317000035</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>OTO BETNOVATE 1+10+5MG/ML SOL OTO FR GTS 10ML</t>
+          <t>PACO 500MG+30MG CX 12 COMP</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H60" s="5" t="n">
-        <v>27</v>
+        <v>24.95</v>
       </c>
       <c r="I60" s="5">
         <f>G60*H60</f>
@@ -4020,13 +4020,13 @@
         <v/>
       </c>
       <c r="K60" s="5" t="n">
-        <v>27</v>
+        <v>31.99</v>
       </c>
       <c r="L60" s="5" t="n">
-        <v>24.82</v>
+        <v>23.0125</v>
       </c>
       <c r="M60" s="5" t="n">
-        <v>25.91556666666667</v>
+        <v>23.99936666666666</v>
       </c>
       <c r="N60" s="6">
         <f>J60/M60-1</f>
@@ -4045,30 +4045,30 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>398941</v>
+        <v>398921</v>
       </c>
       <c r="B61" s="2" t="inlineStr"/>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>7891317000035</t>
+          <t>7891317000042</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>PACO 500MG+30MG CX 12 COMP</t>
+          <t>PACO 500MG+30MG CX 24 COMP</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H61" s="5" t="n">
-        <v>24.95</v>
+        <v>45.32</v>
       </c>
       <c r="I61" s="5">
         <f>G61*H61</f>
@@ -4079,13 +4079,13 @@
         <v/>
       </c>
       <c r="K61" s="5" t="n">
-        <v>31.99</v>
+        <v>46.6</v>
       </c>
       <c r="L61" s="5" t="n">
-        <v>23.0125</v>
+        <v>41.795</v>
       </c>
       <c r="M61" s="5" t="n">
-        <v>23.99936666666666</v>
+        <v>44.73</v>
       </c>
       <c r="N61" s="6">
         <f>J61/M61-1</f>
@@ -4104,30 +4104,30 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>398921</v>
+        <v>644681</v>
       </c>
       <c r="B62" s="2" t="inlineStr"/>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>7891317000042</t>
+          <t>7898031310891</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>PACO 500MG+30MG CX 24 COMP</t>
+          <t>PEDRA HUME SOLUCAO SPRAY 30ML</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H62" s="5" t="n">
-        <v>45.32</v>
+        <v>3.91</v>
       </c>
       <c r="I62" s="5">
         <f>G62*H62</f>
@@ -4138,13 +4138,13 @@
         <v/>
       </c>
       <c r="K62" s="5" t="n">
-        <v>46.6</v>
+        <v>5.45</v>
       </c>
       <c r="L62" s="5" t="n">
-        <v>41.795</v>
+        <v>5.45</v>
       </c>
       <c r="M62" s="5" t="n">
-        <v>44.73</v>
+        <v>5.45</v>
       </c>
       <c r="N62" s="6">
         <f>J62/M62-1</f>
@@ -4163,30 +4163,30 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>644681</v>
+        <v>284281</v>
       </c>
       <c r="B63" s="2" t="inlineStr"/>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>7898031310891</t>
+          <t>7896637025362</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>PEDRA HUME SOLUCAO SPRAY 30ML</t>
+          <t>POSTEC 2,5MG+150UTR POM DERM BG 20G</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>3.91</v>
+        <v>108.14</v>
       </c>
       <c r="I63" s="5">
         <f>G63*H63</f>
@@ -4197,13 +4197,13 @@
         <v/>
       </c>
       <c r="K63" s="5" t="n">
-        <v>5.45</v>
+        <v>108.14</v>
       </c>
       <c r="L63" s="5" t="n">
-        <v>5.45</v>
+        <v>101.2367</v>
       </c>
       <c r="M63" s="5" t="n">
-        <v>5.45</v>
+        <v>103.5378</v>
       </c>
       <c r="N63" s="6">
         <f>J63/M63-1</f>
@@ -4222,30 +4222,30 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>284281</v>
+        <v>500201</v>
       </c>
       <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>7896637025362</t>
+          <t>7897595901309</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>POSTEC 2,5MG+150UTR POM DERM BG 20G</t>
+          <t>PURAN T4 25MCG CX 30 COMP</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>108.14</v>
+        <v>13.36</v>
       </c>
       <c r="I64" s="5">
         <f>G64*H64</f>
@@ -4256,13 +4256,13 @@
         <v/>
       </c>
       <c r="K64" s="5" t="n">
-        <v>108.14</v>
+        <v>13.3467</v>
       </c>
       <c r="L64" s="5" t="n">
-        <v>101.2367</v>
+        <v>11.0783</v>
       </c>
       <c r="M64" s="5" t="n">
-        <v>103.5378</v>
+        <v>12.42</v>
       </c>
       <c r="N64" s="6">
         <f>J64/M64-1</f>
@@ -4274,37 +4274,37 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +0.1% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>500201</v>
+        <v>320861</v>
       </c>
       <c r="B65" s="2" t="inlineStr"/>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>7897595901309</t>
+          <t>7897595901316</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>PURAN T4 25MCG CX 30 COMP</t>
+          <t>PURAN T4 50MCG CX 30 COMP</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H65" s="5" t="n">
-        <v>13.36</v>
+        <v>14.78</v>
       </c>
       <c r="I65" s="5">
         <f>G65*H65</f>
@@ -4315,13 +4315,13 @@
         <v/>
       </c>
       <c r="K65" s="5" t="n">
-        <v>13.3467</v>
+        <v>14.437</v>
       </c>
       <c r="L65" s="5" t="n">
-        <v>11.0783</v>
+        <v>12.2508</v>
       </c>
       <c r="M65" s="5" t="n">
-        <v>12.42</v>
+        <v>13.62703333333333</v>
       </c>
       <c r="N65" s="6">
         <f>J65/M65-1</f>
@@ -4333,37 +4333,37 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.1% vs últ. (≤4%)</t>
+          <t>REAJUSTE +2.4% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>320861</v>
+        <v>14581</v>
       </c>
       <c r="B66" s="2" t="inlineStr"/>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>7897595901316</t>
+          <t>7891106006279</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>PURAN T4 50MCG CX 30 COMP</t>
+          <t>REDOXON 1G TB 10 COMP EFEV SB LARANJA</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>14.78</v>
+        <v>13.47</v>
       </c>
       <c r="I66" s="5">
         <f>G66*H66</f>
@@ -4374,13 +4374,13 @@
         <v/>
       </c>
       <c r="K66" s="5" t="n">
-        <v>14.437</v>
+        <v>13.47</v>
       </c>
       <c r="L66" s="5" t="n">
-        <v>12.2508</v>
+        <v>13.47</v>
       </c>
       <c r="M66" s="5" t="n">
-        <v>13.62703333333333</v>
+        <v>13.47</v>
       </c>
       <c r="N66" s="6">
         <f>J66/M66-1</f>
@@ -4392,37 +4392,37 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +2.4% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>14581</v>
+        <v>565941</v>
       </c>
       <c r="B67" s="2" t="inlineStr"/>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>7891106006279</t>
+          <t>7891106912655</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>REDOXON 1G TB 10 COMP EFEV SB LARANJA</t>
+          <t>REDOXON TRIPLA ACAO 10CP EFERV</t>
         </is>
       </c>
       <c r="E67" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>13.47</v>
+        <v>14.57</v>
       </c>
       <c r="I67" s="5">
         <f>G67*H67</f>
@@ -4433,13 +4433,13 @@
         <v/>
       </c>
       <c r="K67" s="5" t="n">
-        <v>13.47</v>
+        <v>14.155</v>
       </c>
       <c r="L67" s="5" t="n">
-        <v>13.47</v>
+        <v>11.2925</v>
       </c>
       <c r="M67" s="5" t="n">
-        <v>13.47</v>
+        <v>13.1425</v>
       </c>
       <c r="N67" s="6">
         <f>J67/M67-1</f>
@@ -4451,37 +4451,37 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +2.9% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>565941</v>
+        <v>114041</v>
       </c>
       <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>7891106912655</t>
+          <t>7896676432886</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>REDOXON TRIPLA ACAO 10CP EFERV</t>
+          <t>REGENCEL 10000UI+25/5/5MG POM OFT 3,5G</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>14.57</v>
+        <v>12.9</v>
       </c>
       <c r="I68" s="5">
         <f>G68*H68</f>
@@ -4492,13 +4492,13 @@
         <v/>
       </c>
       <c r="K68" s="5" t="n">
-        <v>14.155</v>
+        <v>13.54</v>
       </c>
       <c r="L68" s="5" t="n">
-        <v>11.2925</v>
+        <v>11.94</v>
       </c>
       <c r="M68" s="5" t="n">
-        <v>13.1425</v>
+        <v>12.56333333333333</v>
       </c>
       <c r="N68" s="6">
         <f>J68/M68-1</f>
@@ -4510,37 +4510,37 @@
       </c>
       <c r="P68" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +2.9% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>114041</v>
+        <v>4601</v>
       </c>
       <c r="B69" s="2" t="inlineStr"/>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>7896676432886</t>
+          <t>7891317465667</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>REGENCEL 10000UI+25/5/5MG POM OFT 3,5G</t>
+          <t>SELENE 0,035+2MG CX 21 COMP REV</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="H69" s="5" t="n">
-        <v>12.9</v>
+        <v>26.38</v>
       </c>
       <c r="I69" s="5">
         <f>G69*H69</f>
@@ -4551,13 +4551,13 @@
         <v/>
       </c>
       <c r="K69" s="5" t="n">
-        <v>13.54</v>
+        <v>26.38</v>
       </c>
       <c r="L69" s="5" t="n">
-        <v>11.94</v>
+        <v>24.35</v>
       </c>
       <c r="M69" s="5" t="n">
-        <v>12.56333333333333</v>
+        <v>25.70333333333333</v>
       </c>
       <c r="N69" s="6">
         <f>J69/M69-1</f>
@@ -4576,30 +4576,30 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>4601</v>
+        <v>110341</v>
       </c>
       <c r="B70" s="2" t="inlineStr"/>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>7891317465667</t>
+          <t>7891317421748</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>SELENE 0,035+2MG CX 21 COMP REV</t>
+          <t>SINOT CLAV 875+125MG FR 14 COMP</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="H70" s="5" t="n">
-        <v>26.38</v>
+        <v>59.77</v>
       </c>
       <c r="I70" s="5">
         <f>G70*H70</f>
@@ -4610,13 +4610,13 @@
         <v/>
       </c>
       <c r="K70" s="5" t="n">
-        <v>26.38</v>
+        <v>61.45</v>
       </c>
       <c r="L70" s="5" t="n">
-        <v>24.35</v>
+        <v>59.13</v>
       </c>
       <c r="M70" s="5" t="n">
-        <v>25.70333333333333</v>
+        <v>59.90333333333334</v>
       </c>
       <c r="N70" s="6">
         <f>J70/M70-1</f>
@@ -4635,30 +4635,30 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>110341</v>
+        <v>658381</v>
       </c>
       <c r="B71" s="2" t="inlineStr"/>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>7891317421748</t>
+          <t>7896658020315</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>SINOT CLAV 875+125MG FR 14 COMP</t>
+          <t>SORINE SSC SOL NAS SPRAY 50ML-OUTROS</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H71" s="5" t="n">
-        <v>59.77</v>
+        <v>23.57</v>
       </c>
       <c r="I71" s="5">
         <f>G71*H71</f>
@@ -4669,13 +4669,13 @@
         <v/>
       </c>
       <c r="K71" s="5" t="n">
-        <v>61.45</v>
+        <v>24.75</v>
       </c>
       <c r="L71" s="5" t="n">
-        <v>59.13</v>
+        <v>23.82</v>
       </c>
       <c r="M71" s="5" t="n">
-        <v>59.90333333333334</v>
+        <v>24.13</v>
       </c>
       <c r="N71" s="6">
         <f>J71/M71-1</f>
@@ -4694,30 +4694,30 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>658381</v>
+        <v>645201</v>
       </c>
       <c r="B72" s="2" t="inlineStr"/>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>7896658020315</t>
+          <t>7891317009717</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>SORINE SSC SOL NAS SPRAY 50ML-OUTROS</t>
+          <t>TAMISA NF 0,075+0,030MG CX 21 COMP REV</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H72" s="5" t="n">
-        <v>23.57</v>
+        <v>28.4</v>
       </c>
       <c r="I72" s="5">
         <f>G72*H72</f>
@@ -4728,13 +4728,13 @@
         <v/>
       </c>
       <c r="K72" s="5" t="n">
-        <v>24.75</v>
+        <v>29.1975</v>
       </c>
       <c r="L72" s="5" t="n">
-        <v>23.82</v>
+        <v>26.225</v>
       </c>
       <c r="M72" s="5" t="n">
-        <v>24.13</v>
+        <v>27.875</v>
       </c>
       <c r="N72" s="6">
         <f>J72/M72-1</f>
@@ -4753,30 +4753,30 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>645201</v>
+        <v>345721</v>
       </c>
       <c r="B73" s="2" t="inlineStr"/>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>7891317009717</t>
+          <t>7892953101865</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>TAMISA NF 0,075+0,030MG CX 21 COMP REV</t>
+          <t>TECNOMET 2,5MG CX 20 COMP</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>28.4</v>
+        <v>32.51</v>
       </c>
       <c r="I73" s="5">
         <f>G73*H73</f>
@@ -4787,13 +4787,13 @@
         <v/>
       </c>
       <c r="K73" s="5" t="n">
-        <v>29.1975</v>
+        <v>31.91</v>
       </c>
       <c r="L73" s="5" t="n">
-        <v>26.225</v>
+        <v>27.316</v>
       </c>
       <c r="M73" s="5" t="n">
-        <v>27.875</v>
+        <v>29.852</v>
       </c>
       <c r="N73" s="6">
         <f>J73/M73-1</f>
@@ -4805,37 +4805,37 @@
       </c>
       <c r="P73" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +1.9% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>345721</v>
+        <v>572341</v>
       </c>
       <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>7892953101865</t>
+          <t>7500435171090</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>TECNOMET 2,5MG CX 20 COMP</t>
+          <t>TESTE DE GRAVIDEZ CLEARBLUE DIGIT 1UN</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>32.51</v>
+        <v>38.39</v>
       </c>
       <c r="I74" s="5">
         <f>G74*H74</f>
@@ -4846,13 +4846,13 @@
         <v/>
       </c>
       <c r="K74" s="5" t="n">
-        <v>31.91</v>
+        <v>38.38</v>
       </c>
       <c r="L74" s="5" t="n">
-        <v>27.316</v>
+        <v>37.55</v>
       </c>
       <c r="M74" s="5" t="n">
-        <v>29.852</v>
+        <v>37.55</v>
       </c>
       <c r="N74" s="6">
         <f>J74/M74-1</f>
@@ -4864,24 +4864,24 @@
       </c>
       <c r="P74" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +1.9% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>572341</v>
+        <v>464521</v>
       </c>
       <c r="B75" s="2" t="inlineStr"/>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>7500435171090</t>
+          <t>7896548112717</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>TESTE DE GRAVIDEZ CLEARBLUE DIGIT 1UN</t>
+          <t>TOBREX 3MG SOL OFT FR GTS 5ML</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
@@ -4894,7 +4894,7 @@
         <v>1</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>38.39</v>
+        <v>28.22</v>
       </c>
       <c r="I75" s="5">
         <f>G75*H75</f>
@@ -4905,13 +4905,13 @@
         <v/>
       </c>
       <c r="K75" s="5" t="n">
-        <v>38.38</v>
+        <v>28.09</v>
       </c>
       <c r="L75" s="5" t="n">
-        <v>37.55</v>
+        <v>26.69</v>
       </c>
       <c r="M75" s="5" t="n">
-        <v>37.55</v>
+        <v>27.62333333333333</v>
       </c>
       <c r="N75" s="6">
         <f>J75/M75-1</f>
@@ -4923,37 +4923,37 @@
       </c>
       <c r="P75" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.0% vs últ. (≤4%)</t>
+          <t>REAJUSTE +0.5% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>464521</v>
+        <v>596521</v>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>7896548112717</t>
+          <t>7894916516006</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>TOBREX 3MG SOL OFT FR GTS 5ML</t>
+          <t>TORAGESIC 10MG PEEL OFF CX 10 COMP</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H76" s="5" t="n">
-        <v>28.22</v>
+        <v>26.81</v>
       </c>
       <c r="I76" s="5">
         <f>G76*H76</f>
@@ -4964,13 +4964,13 @@
         <v/>
       </c>
       <c r="K76" s="5" t="n">
-        <v>28.09</v>
+        <v>26.0814</v>
       </c>
       <c r="L76" s="5" t="n">
-        <v>26.69</v>
+        <v>23.048</v>
       </c>
       <c r="M76" s="5" t="n">
-        <v>27.62333333333333</v>
+        <v>23.76266666666666</v>
       </c>
       <c r="N76" s="6">
         <f>J76/M76-1</f>
@@ -4982,37 +4982,37 @@
       </c>
       <c r="P76" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.5% vs últ. (≤4%)</t>
+          <t>REAJUSTE +2.8% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>596521</v>
+        <v>210541</v>
       </c>
       <c r="B77" s="2" t="inlineStr"/>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>7894916516006</t>
+          <t>7891317005931</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>TORAGESIC 10MG PEEL OFF CX 10 COMP</t>
+          <t>TRIMUSK 125+50+300+30MG CX 15 COMP</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="H77" s="5" t="n">
-        <v>26.81</v>
+        <v>17.91</v>
       </c>
       <c r="I77" s="5">
         <f>G77*H77</f>
@@ -5023,13 +5023,13 @@
         <v/>
       </c>
       <c r="K77" s="5" t="n">
-        <v>26.0814</v>
+        <v>17.91</v>
       </c>
       <c r="L77" s="5" t="n">
-        <v>23.048</v>
+        <v>16.955</v>
       </c>
       <c r="M77" s="5" t="n">
-        <v>23.76266666666666</v>
+        <v>17.52833333333333</v>
       </c>
       <c r="N77" s="6">
         <f>J77/M77-1</f>
@@ -5041,37 +5041,37 @@
       </c>
       <c r="P77" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +2.8% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>210541</v>
+        <v>609051</v>
       </c>
       <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>7891317005931</t>
+          <t>7891317025564</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>TRIMUSK 125+50+300+30MG CX 15 COMP</t>
+          <t>TROK 20+0,5MG/G CREM DERM BG 10G</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="H78" s="5" t="n">
-        <v>17.91</v>
+        <v>15</v>
       </c>
       <c r="I78" s="5">
         <f>G78*H78</f>
@@ -5082,13 +5082,13 @@
         <v/>
       </c>
       <c r="K78" s="5" t="n">
-        <v>17.91</v>
+        <v>15.42</v>
       </c>
       <c r="L78" s="5" t="n">
-        <v>16.955</v>
+        <v>14.02</v>
       </c>
       <c r="M78" s="5" t="n">
-        <v>17.52833333333333</v>
+        <v>14.69666666666667</v>
       </c>
       <c r="N78" s="6">
         <f>J78/M78-1</f>
@@ -5107,30 +5107,30 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>609051</v>
+        <v>451941</v>
       </c>
       <c r="B79" s="2" t="inlineStr"/>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>7891317025564</t>
+          <t>7891317445737</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>TROK 20+0,5MG/G CREM DERM BG 10G</t>
+          <t>TROK-N 20+0,5+2,5MG/G CREM DERM BG 30G</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H79" s="5" t="n">
-        <v>15</v>
+        <v>30.98</v>
       </c>
       <c r="I79" s="5">
         <f>G79*H79</f>
@@ -5141,13 +5141,13 @@
         <v/>
       </c>
       <c r="K79" s="5" t="n">
-        <v>15.42</v>
+        <v>31.855</v>
       </c>
       <c r="L79" s="5" t="n">
-        <v>14.02</v>
+        <v>28.9525</v>
       </c>
       <c r="M79" s="5" t="n">
-        <v>14.69666666666667</v>
+        <v>30.34916666666667</v>
       </c>
       <c r="N79" s="6">
         <f>J79/M79-1</f>
@@ -5166,30 +5166,30 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>451941</v>
+        <v>282781</v>
       </c>
       <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>7891317445737</t>
+          <t>7896255717885</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>TROK-N 20+0,5+2,5MG/G CREM DERM BG 30G</t>
+          <t>TROMBOFOB 200UI GEL BG 40G</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H80" s="5" t="n">
-        <v>30.98</v>
+        <v>32.85</v>
       </c>
       <c r="I80" s="5">
         <f>G80*H80</f>
@@ -5200,13 +5200,13 @@
         <v/>
       </c>
       <c r="K80" s="5" t="n">
-        <v>31.855</v>
+        <v>32.62</v>
       </c>
       <c r="L80" s="5" t="n">
-        <v>28.9525</v>
+        <v>25.57</v>
       </c>
       <c r="M80" s="5" t="n">
-        <v>30.34916666666667</v>
+        <v>29.64333333333333</v>
       </c>
       <c r="N80" s="6">
         <f>J80/M80-1</f>
@@ -5218,37 +5218,37 @@
       </c>
       <c r="P80" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
         </is>
       </c>
       <c r="Q80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>282781</v>
+        <v>675881</v>
       </c>
       <c r="B81" s="2" t="inlineStr"/>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>7896255717885</t>
+          <t>7898031310990</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>TROMBOFOB 200UI GEL BG 40G</t>
+          <t>VASELINA LIQUIDA 100ML</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H81" s="5" t="n">
-        <v>32.85</v>
+        <v>3.9</v>
       </c>
       <c r="I81" s="5">
         <f>G81*H81</f>
@@ -5259,13 +5259,13 @@
         <v/>
       </c>
       <c r="K81" s="5" t="n">
-        <v>32.62</v>
+        <v>5.29</v>
       </c>
       <c r="L81" s="5" t="n">
-        <v>25.57</v>
+        <v>5.29</v>
       </c>
       <c r="M81" s="5" t="n">
-        <v>29.64333333333333</v>
+        <v>5.29</v>
       </c>
       <c r="N81" s="6">
         <f>J81/M81-1</f>
@@ -5277,37 +5277,37 @@
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>REAJUSTE +0.7% vs últ. (≤4%)</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>675881</v>
+        <v>219241</v>
       </c>
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>7898031310990</t>
+          <t>7896641813146</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>VASELINA LIQUIDA 100ML</t>
+          <t>VENCIDO - DRAMIN 50 MG CARTELA 10 CP</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H82" s="5" t="n">
-        <v>3.9</v>
+        <v>17.55</v>
       </c>
       <c r="I82" s="5">
         <f>G82*H82</f>
@@ -5317,43 +5317,31 @@
         <f>H82/E82</f>
         <v/>
       </c>
-      <c r="K82" s="5" t="n">
-        <v>5.29</v>
-      </c>
-      <c r="L82" s="5" t="n">
-        <v>5.29</v>
-      </c>
-      <c r="M82" s="5" t="n">
-        <v>5.29</v>
-      </c>
-      <c r="N82" s="6">
-        <f>J82/M82-1</f>
-        <v/>
-      </c>
-      <c r="O82" s="6">
-        <f>J82/K82-1</f>
-        <v/>
-      </c>
+      <c r="K82" s="5" t="n"/>
+      <c r="L82" s="5" t="n"/>
+      <c r="M82" s="5" t="n"/>
+      <c r="N82" s="6" t="n"/>
+      <c r="O82" s="6" t="n"/>
       <c r="P82" s="2" t="inlineStr">
         <is>
-          <t>OK (≤ últ. compra)</t>
+          <t>SEM HISTÓRICO</t>
         </is>
       </c>
       <c r="Q82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>219241</v>
+        <v>461961</v>
       </c>
       <c r="B83" s="2" t="inlineStr"/>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>7896641813146</t>
+          <t>7893454100708</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>VENCIDO - DRAMIN 50 MG CARTELA 10 CP</t>
+          <t>VENCIDO - TIADOL 50MG/G SAB SACO 65G</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
@@ -5366,7 +5354,7 @@
         <v>1</v>
       </c>
       <c r="H83" s="5" t="n">
-        <v>17.55</v>
+        <v>18.4</v>
       </c>
       <c r="I83" s="5">
         <f>G83*H83</f>
@@ -5376,44 +5364,56 @@
         <f>H83/E83</f>
         <v/>
       </c>
-      <c r="K83" s="5" t="n"/>
-      <c r="L83" s="5" t="n"/>
-      <c r="M83" s="5" t="n"/>
-      <c r="N83" s="6" t="n"/>
-      <c r="O83" s="6" t="n"/>
+      <c r="K83" s="5" t="n">
+        <v>19.23</v>
+      </c>
+      <c r="L83" s="5" t="n">
+        <v>19.23</v>
+      </c>
+      <c r="M83" s="5" t="n">
+        <v>19.23</v>
+      </c>
+      <c r="N83" s="6">
+        <f>J83/M83-1</f>
+        <v/>
+      </c>
+      <c r="O83" s="6">
+        <f>J83/K83-1</f>
+        <v/>
+      </c>
       <c r="P83" s="2" t="inlineStr">
         <is>
-          <t>SEM HISTÓRICO</t>
+          <t>OK (≤ últ. compra)</t>
         </is>
       </c>
       <c r="Q83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>461961</v>
+        <v>16681</v>
       </c>
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>7893454100708</t>
+          <t>7898109241485</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>VENCIDO - TIADOL 50MG/G SAB SACO 65G</t>
+          <t>VI-FERRIN 150+0,25+7,5MCG SOL OR FR X 20ML</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H84" s="5" t="n">
-        <v>18.4</v>
+        <v>29.05</v>
       </c>
       <c r="I84" s="5">
         <f>G84*H84</f>
@@ -5424,13 +5424,13 @@
         <v/>
       </c>
       <c r="K84" s="5" t="n">
-        <v>19.23</v>
+        <v>29.05</v>
       </c>
       <c r="L84" s="5" t="n">
-        <v>19.23</v>
+        <v>29.05</v>
       </c>
       <c r="M84" s="5" t="n">
-        <v>19.23</v>
+        <v>29.05</v>
       </c>
       <c r="N84" s="6">
         <f>J84/M84-1</f>
@@ -5449,30 +5449,30 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>16681</v>
+        <v>993</v>
       </c>
       <c r="B85" s="2" t="inlineStr"/>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>7898109241485</t>
+          <t>75075644</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>VI-FERRIN 150+0,25+7,5MCG SOL OR FR X 20ML</t>
+          <t>VICK BABY RUB 12G LATA</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H85" s="5" t="n">
-        <v>29.05</v>
+        <v>92.44000000000001</v>
       </c>
       <c r="I85" s="5">
         <f>G85*H85</f>
@@ -5483,13 +5483,13 @@
         <v/>
       </c>
       <c r="K85" s="5" t="n">
-        <v>29.05</v>
+        <v>15.8375</v>
       </c>
       <c r="L85" s="5" t="n">
-        <v>29.05</v>
+        <v>13.1538</v>
       </c>
       <c r="M85" s="5" t="n">
-        <v>29.05</v>
+        <v>14.94293333333333</v>
       </c>
       <c r="N85" s="6">
         <f>J85/M85-1</f>
@@ -5504,31 +5504,35 @@
           <t>OK (≤ últ. compra)</t>
         </is>
       </c>
-      <c r="Q85" s="2" t="inlineStr"/>
+      <c r="Q85" s="2" t="inlineStr">
+        <is>
+          <t>1 emb = 6 un</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>993</v>
+        <v>600581</v>
       </c>
       <c r="B86" s="2" t="inlineStr"/>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>75075644</t>
+          <t>7501001246730</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>VICK BABY RUB 12G LATA</t>
+          <t>VICK LATINHA 12G</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H86" s="5" t="n">
         <v>92.44000000000001</v>
@@ -5542,13 +5546,13 @@
         <v/>
       </c>
       <c r="K86" s="5" t="n">
-        <v>15.8375</v>
+        <v>17.0408</v>
       </c>
       <c r="L86" s="5" t="n">
-        <v>13.1538</v>
+        <v>11.9136</v>
       </c>
       <c r="M86" s="5" t="n">
-        <v>14.94293333333333</v>
+        <v>14.19566666666667</v>
       </c>
       <c r="N86" s="6">
         <f>J86/M86-1</f>
@@ -5565,36 +5569,36 @@
       </c>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>1 emb = 6 un</t>
+          <t>preços divergentes entre EANs (usado menor); 1 emb = 24 un; conferir emb.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>600581</v>
+        <v>542821</v>
       </c>
       <c r="B87" s="2" t="inlineStr"/>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>7501001246730</t>
+          <t>789112444</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>VICK LATINHA 12G</t>
+          <t>VICK VAPORUB 30G POTE</t>
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H87" s="5" t="n">
-        <v>92.44000000000001</v>
+        <v>36.32</v>
       </c>
       <c r="I87" s="5">
         <f>G87*H87</f>
@@ -5605,13 +5609,13 @@
         <v/>
       </c>
       <c r="K87" s="5" t="n">
-        <v>17.0408</v>
+        <v>38.6</v>
       </c>
       <c r="L87" s="5" t="n">
-        <v>11.9136</v>
+        <v>28.35</v>
       </c>
       <c r="M87" s="5" t="n">
-        <v>14.19566666666667</v>
+        <v>32.6096</v>
       </c>
       <c r="N87" s="6">
         <f>J87/M87-1</f>
@@ -5626,38 +5630,34 @@
           <t>OK (≤ últ. compra)</t>
         </is>
       </c>
-      <c r="Q87" s="2" t="inlineStr">
-        <is>
-          <t>preços divergentes entre EANs (usado menor); 1 emb = 24 un; conferir emb.</t>
-        </is>
-      </c>
+      <c r="Q87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>542821</v>
+        <v>254901</v>
       </c>
       <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>789112444</t>
+          <t>7896548197554</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>VICK VAPORUB 30G POTE</t>
+          <t>VIGADEXA 5+1MG/ML SOL OFT FR GOT 5ML</t>
         </is>
       </c>
       <c r="E88" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H88" s="5" t="n">
-        <v>36.32</v>
+        <v>38.7</v>
       </c>
       <c r="I88" s="5">
         <f>G88*H88</f>
@@ -5668,13 +5668,13 @@
         <v/>
       </c>
       <c r="K88" s="5" t="n">
-        <v>38.6</v>
+        <v>50.5</v>
       </c>
       <c r="L88" s="5" t="n">
-        <v>28.35</v>
+        <v>35.1083</v>
       </c>
       <c r="M88" s="5" t="n">
-        <v>32.6096</v>
+        <v>36.87476666666667</v>
       </c>
       <c r="N88" s="6">
         <f>J88/M88-1</f>
@@ -5693,30 +5693,30 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>254901</v>
+        <v>532061</v>
       </c>
       <c r="B89" s="2" t="inlineStr"/>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>7896548197554</t>
+          <t>7894164006014</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>VIGADEXA 5+1MG/ML SOL OFT FR GOT 5ML</t>
+          <t>VITAXON C TRIPLA ACAO EFERVECE CX C/ 10 CP</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>1</v>
+        <v>62</v>
       </c>
       <c r="H89" s="5" t="n">
-        <v>38.7</v>
+        <v>4.58</v>
       </c>
       <c r="I89" s="5">
         <f>G89*H89</f>
@@ -5727,13 +5727,13 @@
         <v/>
       </c>
       <c r="K89" s="5" t="n">
-        <v>50.5</v>
+        <v>4.58</v>
       </c>
       <c r="L89" s="5" t="n">
-        <v>35.1083</v>
+        <v>4.58</v>
       </c>
       <c r="M89" s="5" t="n">
-        <v>36.87476666666667</v>
+        <v>4.58</v>
       </c>
       <c r="N89" s="6">
         <f>J89/M89-1</f>
@@ -5751,77 +5751,18 @@
       <c r="Q89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>532061</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr"/>
-      <c r="C90" s="3" t="inlineStr">
-        <is>
-          <t>7894164006014</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>VITAXON C TRIPLA ACAO EFERVECE CX C/ 10 CP</t>
-        </is>
-      </c>
-      <c r="E90" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F90" s="4" t="n">
-        <v>62</v>
-      </c>
-      <c r="G90" s="4" t="n">
-        <v>62</v>
-      </c>
-      <c r="H90" s="5" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="I90" s="5">
-        <f>G90*H90</f>
-        <v/>
-      </c>
-      <c r="J90" s="5">
-        <f>H90/E90</f>
-        <v/>
-      </c>
-      <c r="K90" s="5" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="L90" s="5" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="M90" s="5" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="N90" s="6">
-        <f>J90/M90-1</f>
-        <v/>
-      </c>
-      <c r="O90" s="6">
-        <f>J90/K90-1</f>
-        <v/>
-      </c>
-      <c r="P90" s="2" t="inlineStr">
-        <is>
-          <t>OK (≤ últ. compra)</t>
-        </is>
-      </c>
-      <c r="Q90" s="2" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="I91" s="8">
-        <f>SUM(I2:I90)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="9" t="inlineStr">
+      <c r="I90" s="8">
+        <f>SUM(I2:I89)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="inlineStr">
         <is>
           <t>Pedido FINAL TAPAJOS — cotação 08/09/2026 (fechada 09/09). Somente itens aprovados: teto de reajuste de 4% sobre a última compra OU 6% sobre a média histórica (3/6/12m). 'Qtd pedido' na embalagem do fornecedor.</t>
         </is>

</xml_diff>